<commit_message>
Rôles validés (9), source du poids article, décisions mises à jour
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/PARAMETRES_SOP.xlsx
+++ b/modeles/xlsx/PARAMETRES_SOP.xlsx
@@ -621,80 +621,80 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qui corrige la prévision des TC</t>
+          <t xml:space="preserve">Rôles</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Responsable de territoire, à confirmer selon le modèle</t>
+          <t xml:space="preserve">ADMIN, PREV, RM, AM, RT, CD, RBP, TC, SUPPLY</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maille des corrections</t>
+          <t xml:space="preserve">Qui corrige la prévision des TC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Article</t>
+          <t xml:space="preserve">Responsable de territoire, à confirmer selon le modèle</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
+          <t xml:space="preserve">A_VALIDER</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rattachement semaine vers mois</t>
+          <t xml:space="preserve">Maille des corrections</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mois du jeudi</t>
+          <t xml:space="preserve">Article</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROPOSITION</t>
+          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poids article</t>
+          <t xml:space="preserve">Rattachement semaine vers mois</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Système source à identifier</t>
+          <t xml:space="preserve">Mois du jeudi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">A_COMPLETER</t>
+          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accès au budget</t>
+          <t xml:space="preserve">Poids article</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">À valider avec Emmanuel</t>
+          <t xml:space="preserve">Lu dans un Google Sheet, lien à fournir</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -706,15 +706,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Accès au budget</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">À valider avec Emmanuel</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A_COMPLETER</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Dates des campagnes PAC1 à PAC4 et morte saison</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t xml:space="preserve">À renseigner</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t xml:space="preserve">A_COMPLETER</t>
         </is>
@@ -1602,110 +1619,6 @@
       <c r="J10" t="inlineStr">
         <is>
           <t xml:space="preserve">GLOBAL ou périmètre explicite</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CDG</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OUI</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OUI</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GLOBAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DIR</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OUI</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OUI</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GLOBAL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruptures : vue demande et vue réel en parallèle
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/PARAMETRES_SOP.xlsx
+++ b/modeles/xlsx/PARAMETRES_SOP.xlsx
@@ -1104,12 +1104,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dates des campagnes PAC1 à PAC4 et morte saison</t>
+          <t xml:space="preserve">Traitement par défaut des ventes en rupture</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">À renseigner</t>
+          <t xml:space="preserve">Perdues, reportées ou substituées : à décider, modifiable pour chaque rupture</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1121,49 +1121,66 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grain hebdomadaire de la prévision</t>
+          <t xml:space="preserve">Dates des campagnes PAC1 à PAC4 et morte saison</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mois pour le comité, semaine en stockage et publication</t>
+          <t xml:space="preserve">À renseigner</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">A_VALIDER</t>
+          <t xml:space="preserve">A_COMPLETER</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date de référence des ventes</t>
+          <t xml:space="preserve">Grain hebdomadaire de la prévision</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date de livraison ou de commande à choisir</t>
+          <t xml:space="preserve">Mois pour le comité, semaine en stockage et publication</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">A_COMPLETER</t>
+          <t xml:space="preserve">A_VALIDER</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Date de référence des ventes</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date de livraison ou de commande à choisir</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A_COMPLETER</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t xml:space="preserve">Priorité entre les sources de poids</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t xml:space="preserve">Poids de réf, Poids brut, Poids unitaire</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t xml:space="preserve">A_COMPLETER</t>
         </is>

</xml_diff>

<commit_message>
Cadençage à la semaine : coefficients hebdomadaires, prévision stockée sur l'horizon, ajustements par semaine
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/PARAMETRES_SOP.xlsx
+++ b/modeles/xlsx/PARAMETRES_SOP.xlsx
@@ -415,13 +415,12 @@
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,35 +446,30 @@
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Granularite</t>
+          <t xml:space="preserve">Semaine</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Periode</t>
+          <t xml:space="preserve">Coefficient</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Coefficient</t>
+          <t xml:space="preserve">Origine</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Origine</t>
+          <t xml:space="preserve">Version coefficients</t>
         </is>
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Version coefficients</t>
+          <t xml:space="preserve">Validation</t>
         </is>
       </c>
       <c r="J1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Validation</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Valide par</t>
         </is>
@@ -1138,17 +1132,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grain hebdomadaire de la prévision</t>
+          <t xml:space="preserve">Cadençage</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mois pour le comité, semaine en stockage et publication</t>
+          <t xml:space="preserve">À la semaine (semaine ISO). Les mois du comité s'obtiennent en additionnant les semaines</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
         </is>
       </c>
     </row>
@@ -1371,32 +1365,83 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HORIZON_HEBDO_SEMAINES</t>
+          <t xml:space="preserve">PONDERATION_ANNEES</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">78</t>
+          <t xml:space="preserve">50/30/20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aligné sur le suivi de stock actuel (S32 2025 à S26 2027)</t>
+          <t xml:space="preserve">Poids de N-1, N-2, N-3 dans la moyenne pondérée (à valider)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t xml:space="preserve">ALPHA_LISSAGE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0,3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lissage exponentiel (à valider)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUBLICATION_HEBDO_TOUS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI = publier tous les articles à la semaine, sinon ceux de PARAMETRES_STOCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HORIZON_HEBDO_SEMAINES</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aligné sur le suivi de stock actuel (S32 2025 à S26 2027)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t xml:space="preserve">RATTACHEMENT_SEMAINE</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t xml:space="preserve">JEUDI</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t xml:space="preserve">Une semaine appartient au mois de son jeudi (à confirmer)</t>
         </is>

</xml_diff>

<commit_message>
Capacités par plateforme et famille, plan d'approvisionnement cadencé
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/PARAMETRES_SOP.xlsx
+++ b/modeles/xlsx/PARAMETRES_SOP.xlsx
@@ -12,17 +12,18 @@
     <sheet name="GAMME" sheetId="8" r:id="rId8"/>
     <sheet name="SUBSTITUTIONS" sheetId="9" r:id="rId9"/>
     <sheet name="PLATEFORMES" sheetId="10" r:id="rId10"/>
-    <sheet name="AFFECTATION_PLATEFORME" sheetId="11" r:id="rId11"/>
-    <sheet name="FORCAGES" sheetId="12" r:id="rId12"/>
-    <sheet name="POINTS" sheetId="13" r:id="rId13"/>
-    <sheet name="CALENDRIER" sheetId="14" r:id="rId14"/>
-    <sheet name="COEFFICIENTS" sheetId="15" r:id="rId15"/>
-    <sheet name="CONTRAINTES_APPRO" sheetId="16" r:id="rId16"/>
-    <sheet name="ROUTES_APPRO" sheetId="17" r:id="rId17"/>
-    <sheet name="PARAMETRES_STOCK" sheetId="18" r:id="rId18"/>
-    <sheet name="SEUILS_ALERTES" sheetId="19" r:id="rId19"/>
-    <sheet name="SOURCES" sheetId="20" r:id="rId20"/>
-    <sheet name="ARBITRAGES" sheetId="21" r:id="rId21"/>
+    <sheet name="CAPACITES" sheetId="11" r:id="rId11"/>
+    <sheet name="AFFECTATION_PLATEFORME" sheetId="12" r:id="rId12"/>
+    <sheet name="FORCAGES" sheetId="13" r:id="rId13"/>
+    <sheet name="POINTS" sheetId="14" r:id="rId14"/>
+    <sheet name="CALENDRIER" sheetId="15" r:id="rId15"/>
+    <sheet name="COEFFICIENTS" sheetId="16" r:id="rId16"/>
+    <sheet name="CONTRAINTES_APPRO" sheetId="17" r:id="rId17"/>
+    <sheet name="ROUTES_APPRO" sheetId="18" r:id="rId18"/>
+    <sheet name="PARAMETRES_STOCK" sheetId="19" r:id="rId19"/>
+    <sheet name="SEUILS_ALERTES" sheetId="20" r:id="rId20"/>
+    <sheet name="SOURCES" sheetId="21" r:id="rId21"/>
+    <sheet name="ARBITRAGES" sheetId="22" r:id="rId22"/>
   </sheets>
 </workbook>
 </file>
@@ -134,9 +135,6 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -166,21 +164,6 @@
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Capacite T</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Stock mini T</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Stock maxi T</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Actif</t>
         </is>
@@ -191,6 +174,77 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="25" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Plateforme</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Niveau</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Cle niveau</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Type capacite</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Unite</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Capacite</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Seuil alerte pourcent</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Debut validite</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Fin validite</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Commentaire</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -243,7 +297,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -308,7 +362,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -361,7 +415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -408,7 +462,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -479,7 +533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -491,9 +545,11 @@
     <col min="7" max="7" width="19" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
     <col min="9" max="9" width="19" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
+    <col min="11" max="11" width="23" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,15 +600,25 @@
       </c>
       <c r="J1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Avance max semaines</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Retard max semaines</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Debut validite</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="1">
+      <c r="M1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Fin validite</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="1">
+      <c r="N1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Commentaire</t>
         </is>
@@ -562,7 +628,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -621,7 +687,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -659,59 +725,6 @@
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Actif</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="21" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Code alerte</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Libelle</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Seuil</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Unite seuil</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Perimetre</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Role destinataire</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Actif</t>
         </is>
@@ -871,6 +884,59 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Code alerte</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Libelle</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Seuil</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Unite seuil</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Perimetre</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Role destinataire</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Actif</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
@@ -951,7 +1017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1115,12 +1181,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dates des campagnes PAC1 à PAC4 et morte saison</t>
+          <t xml:space="preserve">Unité des capacités</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">À renseigner</t>
+          <t xml:space="preserve">Tonnes, palettes ou m³ selon la plateforme, à préciser</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1132,29 +1198,29 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cadençage</t>
+          <t xml:space="preserve">Capacités par plateforme seule ou aussi par famille</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">À la semaine (semaine ISO). Les mois du comité s'obtiennent en additionnant les semaines</t>
+          <t xml:space="preserve">Les deux sont prévus dans CAPACITES</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
+          <t xml:space="preserve">A_VALIDER</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date de référence des ventes</t>
+          <t xml:space="preserve">Décalage autorisé d'une commande</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date de livraison ou de commande à choisir</t>
+          <t xml:space="preserve">Avance et retard maximum par fournisseur et article</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1166,15 +1232,66 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t xml:space="preserve">Dates des campagnes PAC1 à PAC4 et morte saison</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">À renseigner</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A_COMPLETER</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cadençage</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">À la semaine (semaine ISO). Les mois du comité s'obtiennent en additionnant les semaines</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date de référence des ventes</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date de livraison ou de commande à choisir</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A_COMPLETER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t xml:space="preserve">Priorité entre les sources de poids</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t xml:space="preserve">Poids de réf, Poids brut, Poids unitaire</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t xml:space="preserve">A_COMPLETER</t>
         </is>
@@ -2172,16 +2289,17 @@
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="16" customWidth="1"/>
-    <col min="16" max="16" width="15" customWidth="1"/>
-    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="17" customWidth="1"/>
+    <col min="16" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="15" customWidth="1"/>
     <col min="18" max="18" width="14" customWidth="1"/>
-    <col min="19" max="19" width="15" customWidth="1"/>
-    <col min="20" max="20" width="19" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="19" customWidth="1"/>
-    <col min="22" max="22" width="14" customWidth="1"/>
-    <col min="23" max="23" width="15" customWidth="1"/>
+    <col min="22" max="22" width="19" customWidth="1"/>
+    <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="24" max="24" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2252,50 +2370,55 @@
       </c>
       <c r="N1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Unites par palette</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Poids article</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr" s="1">
+      <c r="P1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Source poids</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="1">
+      <c r="Q1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Unite poids</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="1">
+      <c r="R1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Densite</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="1">
+      <c r="S1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Dose ha</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr" s="1">
+      <c r="T1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Coefficient</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr" s="1">
+      <c r="U1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Mode conversion</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr" s="1">
+      <c r="V1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Date fin de vie</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr" s="1">
+      <c r="W1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Actif</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr" s="1">
+      <c r="X1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Commentaire</t>
         </is>

</xml_diff>

<commit_message>
Zones, articles dangereux, unités L/kg/T/U, décideurs et demandes de décalage ; écran Approvisionnements
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/PARAMETRES_SOP.xlsx
+++ b/modeles/xlsx/PARAMETRES_SOP.xlsx
@@ -13,17 +13,19 @@
     <sheet name="SUBSTITUTIONS" sheetId="9" r:id="rId9"/>
     <sheet name="PLATEFORMES" sheetId="10" r:id="rId10"/>
     <sheet name="CAPACITES" sheetId="11" r:id="rId11"/>
-    <sheet name="AFFECTATION_PLATEFORME" sheetId="12" r:id="rId12"/>
-    <sheet name="FORCAGES" sheetId="13" r:id="rId13"/>
-    <sheet name="POINTS" sheetId="14" r:id="rId14"/>
-    <sheet name="CALENDRIER" sheetId="15" r:id="rId15"/>
-    <sheet name="COEFFICIENTS" sheetId="16" r:id="rId16"/>
-    <sheet name="CONTRAINTES_APPRO" sheetId="17" r:id="rId17"/>
-    <sheet name="ROUTES_APPRO" sheetId="18" r:id="rId18"/>
-    <sheet name="PARAMETRES_STOCK" sheetId="19" r:id="rId19"/>
-    <sheet name="SEUILS_ALERTES" sheetId="20" r:id="rId20"/>
-    <sheet name="SOURCES" sheetId="21" r:id="rId21"/>
-    <sheet name="ARBITRAGES" sheetId="22" r:id="rId22"/>
+    <sheet name="REGLES_STOCKAGE" sheetId="12" r:id="rId12"/>
+    <sheet name="AFFECTATION_PLATEFORME" sheetId="13" r:id="rId13"/>
+    <sheet name="FORCAGES" sheetId="14" r:id="rId14"/>
+    <sheet name="POINTS" sheetId="15" r:id="rId15"/>
+    <sheet name="CALENDRIER" sheetId="16" r:id="rId16"/>
+    <sheet name="COEFFICIENTS" sheetId="17" r:id="rId17"/>
+    <sheet name="CONTRAINTES_APPRO" sheetId="18" r:id="rId18"/>
+    <sheet name="DECIDEURS_APPRO" sheetId="19" r:id="rId19"/>
+    <sheet name="ROUTES_APPRO" sheetId="20" r:id="rId20"/>
+    <sheet name="PARAMETRES_STOCK" sheetId="21" r:id="rId21"/>
+    <sheet name="SEUILS_ALERTES" sheetId="22" r:id="rId22"/>
+    <sheet name="SOURCES" sheetId="23" r:id="rId23"/>
+    <sheet name="ARBITRAGES" sheetId="24" r:id="rId24"/>
   </sheets>
 </workbook>
 </file>
@@ -169,6 +171,99 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GLOMEL</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Glomel</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATEFORME</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CEVEZO2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cevezo 2 (Glomel)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZONE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GLOMEL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GRUEL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gruel</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATEFORME</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAMPENEAC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Campénéac</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLATEFORME</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -248,6 +343,85 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Plateforme</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Zone</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Critere</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Valeur critere</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Mode</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Actif</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GLOMEL</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CEVEZO2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DANGEREUX</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OBLIGATOIRE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
@@ -297,7 +471,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -362,7 +536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -415,7 +589,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -462,7 +636,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -533,7 +707,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -628,103 +802,50 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Type campagne</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Marche</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Plateforme</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Code produit</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Marche</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Type source</t>
+          <t xml:space="preserve">Email Google</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Code source</t>
+          <t xml:space="preserve">Pouvoir</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Delai semaines</t>
+          <t xml:space="preserve">Origine represente</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Actif</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Commentaire</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Plateforme</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Code produit</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Stock mini</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Stock cible</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Lot reappro</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Actif</t>
         </is>
@@ -884,6 +1005,112 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Plateforme</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Code produit</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Marche</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Type source</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Code source</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Delai semaines</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Actif</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Commentaire</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Plateforme</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Code produit</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Stock mini</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Stock cible</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Lot reappro</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Actif</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
@@ -934,7 +1161,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1017,7 +1244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1186,41 +1413,41 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tonnes, palettes ou m³ selon la plateforme, à préciser</t>
+          <t xml:space="preserve">Tonnes, kg, litres ou unités selon la plateforme et la famille</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">A_COMPLETER</t>
+          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capacités par plateforme seule ou aussi par famille</t>
+          <t xml:space="preserve">Niveau des capacités</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les deux sont prévus dans CAPACITES</t>
+          <t xml:space="preserve">Plateforme, zone (ex. Cevezo 2 à Glomel), famille, article dangereux</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">A_VALIDER</t>
+          <t xml:space="preserve">VALIDE_UTILISATEUR</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Décalage autorisé d'une commande</t>
+          <t xml:space="preserve">Décalage d'une commande</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avance et retard maximum par fournisseur et article</t>
+          <t xml:space="preserve">Plusieurs décideurs selon la période PAC, demande du client ou de la logistique (DECIDEURS_APPRO). Noms à fournir</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2289,17 +2516,18 @@
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="15" width="17" customWidth="1"/>
-    <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="15" customWidth="1"/>
-    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="16" max="16" width="17" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="15" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="15" customWidth="1"/>
-    <col min="21" max="21" width="19" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="15" customWidth="1"/>
     <col min="22" max="22" width="19" customWidth="1"/>
-    <col min="23" max="23" width="14" customWidth="1"/>
-    <col min="24" max="24" width="15" customWidth="1"/>
+    <col min="23" max="23" width="19" customWidth="1"/>
+    <col min="24" max="24" width="14" customWidth="1"/>
+    <col min="25" max="25" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2370,55 +2598,60 @@
       </c>
       <c r="N1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Unites par palette</t>
+          <t xml:space="preserve">Dangereux</t>
         </is>
       </c>
       <c r="O1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Classe danger</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Poids article</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="1">
+      <c r="Q1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Source poids</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="1">
+      <c r="R1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Unite poids</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="1">
+      <c r="S1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Densite</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr" s="1">
+      <c r="T1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Dose ha</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr" s="1">
+      <c r="U1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Coefficient</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr" s="1">
+      <c r="V1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Mode conversion</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr" s="1">
+      <c r="W1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Date fin de vie</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr" s="1">
+      <c r="X1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Actif</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr" s="1">
+      <c r="Y1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Commentaire</t>
         </is>

</xml_diff>

<commit_message>
Historique des ventes d'un PAC lu depuis les fichiers déclarés dans SOURCES (modèle v0.8)
SOURCES gagne la nature HISTO_PAC et les colonnes ID campagne, Entite, PAC, Annees, Format.
Nouvel écran Historique, lecture par onglet Données AAAA, droits limités au code TC et à l'entité,
contrôles de mise en service des onglets et des colonnes. 68 tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/PARAMETRES_SOP.xlsx
+++ b/modeles/xlsx/PARAMETRES_SOP.xlsx
@@ -96,7 +96,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modèle de structure v0.7 – à compléter. L'application contrôle que les onglets et colonnes correspondent à cette version.</t>
+          <t xml:space="preserve">Modèle de structure v0.8 – à compléter. L'application contrôle que les onglets et colonnes correspondent à cette version.</t>
         </is>
       </c>
     </row>
@@ -1176,6 +1176,11 @@
     <col min="10" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1237,6 +1242,155 @@
       <c r="L1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Commentaire</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ID campagne</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Entite</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">PAC</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Annees</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Format</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HISTO_EUREDEN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HISTO_PAC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Données {ANNEE}</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A_LA_DEMANDE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QLIK</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coller l'ID du fichier, puis Actif import = OUI</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coop EUREDEN</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PAC1</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024,2025,2026</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SHEETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HISTO_ONA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HISTO_PAC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Données {ANNEE}</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A_LA_DEMANDE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QLIK</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coller l'ID du fichier, puis Actif import = OUI</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NEGOCE ONA</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PAC1</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024,2025,2026</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SHEETS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Catalogue (marché, famille, unité) lu dans la sortie EurePrev : vue par marché, cadençage par marché, unités de stock et tonnes en KG
Guide de mise en service. 197 tests unitaires et 23 étapes de bout en bout.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VDUD2te9mLDL4jRRkQGkWq
</commit_message>
<xml_diff>
--- a/modeles/xlsx/PARAMETRES_SOP.xlsx
+++ b/modeles/xlsx/PARAMETRES_SOP.xlsx
@@ -1880,66 +1880,95 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALPHA_LISSAGE</t>
+          <t xml:space="preserve">BASE_ARBITRAGE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">0,3</t>
+          <t xml:space="preserve">STATISTIQUE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lissage exponentiel (à valider)</t>
+          <t xml:space="preserve">Quantité de départ de l'arbitrage : STATISTIQUE ou TC (saisie des TC quand elle existe)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PUBLICATION_HEBDO_TOUS</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NON</t>
+          <t xml:space="preserve">BUDGET_VERSION</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">OUI = publier tous les articles à la semaine, sinon ceux de PARAMETRES_STOCK</t>
+          <t xml:space="preserve">Version du budget à comparer. Vide = dernière version du fichier</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HORIZON_HEBDO_SEMAINES</t>
+          <t xml:space="preserve">ALPHA_LISSAGE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">78</t>
+          <t xml:space="preserve">0,3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aligné sur le suivi de stock actuel (S32 2025 à S26 2027)</t>
+          <t xml:space="preserve">Lissage exponentiel (à valider)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t xml:space="preserve">PUBLICATION_HEBDO_TOUS</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NON</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OUI = publier tous les articles à la semaine, sinon ceux de PARAMETRES_STOCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HORIZON_HEBDO_SEMAINES</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aligné sur le suivi de stock actuel (S32 2025 à S26 2027)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t xml:space="preserve">RATTACHEMENT_SEMAINE</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t xml:space="preserve">JEUDI</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t xml:space="preserve">Une semaine appartient au mois de son jeudi (à confirmer)</t>
         </is>

</xml_diff>